<commit_message>
UX: widen business_profile column (2x), convert <br> literals to line breaks
</commit_message>
<xml_diff>
--- a/jobs_master.xlsx
+++ b/jobs_master.xlsx
@@ -646,8 +646,8 @@
     <col width="30" customWidth="1" min="14" max="14"/>
     <col width="50" customWidth="1" min="15" max="15"/>
     <col width="32" customWidth="1" min="16" max="16"/>
-    <col width="32" customWidth="1" min="17" max="17"/>
-    <col width="32" customWidth="1" min="18" max="18"/>
+    <col width="65" customWidth="1" min="17" max="17"/>
+    <col width="50" customWidth="1" min="18" max="18"/>
     <col width="30" customWidth="1" min="19" max="19"/>
     <col width="8" customWidth="1" min="20" max="20"/>
   </cols>
@@ -3667,7 +3667,14 @@
       </c>
       <c r="Q37" s="4" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R37" s="4" t="inlineStr">
@@ -3753,7 +3760,14 @@
       </c>
       <c r="Q38" s="5" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R38" s="5" t="inlineStr">
@@ -3839,7 +3853,14 @@
       </c>
       <c r="Q39" s="5" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R39" s="5" t="inlineStr">
@@ -3925,7 +3946,14 @@
       </c>
       <c r="Q40" s="5" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R40" s="5" t="inlineStr">
@@ -4011,7 +4039,14 @@
       </c>
       <c r="Q41" s="6" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R41" s="6" t="inlineStr">
@@ -4097,7 +4132,14 @@
       </c>
       <c r="Q42" s="6" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R42" s="6" t="inlineStr">
@@ -4183,7 +4225,14 @@
       </c>
       <c r="Q43" s="6" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R43" s="6" t="inlineStr">
@@ -4269,7 +4318,14 @@
       </c>
       <c r="Q44" s="6" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R44" s="6" t="inlineStr">
@@ -4355,7 +4411,14 @@
       </c>
       <c r="Q45" s="6" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R45" s="6" t="inlineStr">
@@ -4441,7 +4504,14 @@
       </c>
       <c r="Q46" s="6" t="inlineStr">
         <is>
-          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий&lt;br&gt;- Ведется работа с детьми (минимум 3 занятия в неделю)&lt;br&gt;- Активных клиентов около 200, с сезонным ростом после лета&lt;br&gt;- Важна автоматизация зарплат тренеров и администраторов&lt;br&gt;- Используется мобильное приложение для клиентов и тренеров&lt;br&gt;- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)&lt;br&gt;- Важна интеграция с CRM и автоматизация процессов&lt;br&gt;- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
+          <t>Тип бизнеса: Студия, предоставляющая групповые и персональные занятия (в том числе хореография), фитнес-услуги | Особенности бизнеса: - Есть услуги (пакеты услуг) и абонементы (обычно групповые занятия) с ограничением по времени и количеству занятий
+- Ведется работа с детьми (минимум 3 занятия в неделю)
+- Активных клиентов около 200, с сезонным ростом после лета
+- Важна автоматизация зарплат тренеров и администраторов
+- Используется мобильное приложение для клиентов и тренеров
+- Ведется коммуникация с родителями через мессенджеры и соцсети (WhatsApp, ВКонтакте, Instagram)
+- Важна интеграция с CRM и автоматизация процессов
+- Есть потребность в удобном управлении персональными занятиями и расписанием тренеров</t>
         </is>
       </c>
       <c r="R46" s="6" t="inlineStr">
@@ -4531,7 +4601,14 @@
       </c>
       <c r="Q47" s="4" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R47" s="4" t="inlineStr">
@@ -4621,7 +4698,14 @@
       </c>
       <c r="Q48" s="5" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R48" s="5" t="inlineStr">
@@ -4711,7 +4795,14 @@
       </c>
       <c r="Q49" s="5" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R49" s="5" t="inlineStr">
@@ -4801,7 +4892,14 @@
       </c>
       <c r="Q50" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R50" s="6" t="inlineStr">
@@ -4891,7 +4989,14 @@
       </c>
       <c r="Q51" s="5" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R51" s="5" t="inlineStr">
@@ -4981,7 +5086,14 @@
       </c>
       <c r="Q52" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
@@ -5067,7 +5179,14 @@
       </c>
       <c r="Q53" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R53" s="6" t="inlineStr">
@@ -5153,7 +5272,14 @@
       </c>
       <c r="Q54" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R54" s="6" t="inlineStr">
@@ -5239,7 +5365,14 @@
       </c>
       <c r="Q55" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R55" s="6" t="inlineStr">
@@ -5325,7 +5458,14 @@
       </c>
       <c r="Q56" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R56" s="6" t="inlineStr">
@@ -5411,7 +5551,14 @@
       </c>
       <c r="Q57" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R57" s="6" t="inlineStr">
@@ -5497,7 +5644,14 @@
       </c>
       <c r="Q58" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R58" s="6" t="inlineStr">
@@ -5583,7 +5737,14 @@
       </c>
       <c r="Q59" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R59" s="6" t="inlineStr">
@@ -5669,7 +5830,14 @@
       </c>
       <c r="Q60" s="6" t="inlineStr">
         <is>
-          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) &lt;br&gt; - Оплата раз в 4 недели &lt;br&gt; - Есть дети и взрослые &lt;br&gt; - Родители оплачивают за детей &lt;br&gt; - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp &lt;br&gt; - Используют налог на профессиональный доход (самозанятые), планируют переход на патент &lt;br&gt; - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel &lt;br&gt; - Планируют расширение команды</t>
+          <t>Бизнес: Танцевальная школа/студия с детскими и взрослыми группами, ансамбль, 9 классов, групповые занятия по расписанию, фиксированная оплата за период (4 недели), а также планируются персональные тренировки. | Особенности бизнеса: - Групповые занятия по расписанию (классы ходят целым составом весь год) 
+ - Оплата раз в 4 недели 
+ - Есть дети и взрослые 
+ - Родители оплачивают за детей 
+ - Нет сайта, есть группа ВКонтакте, Telegram, WhatsApp 
+ - Используют налог на профессиональный доход (самозанятые), планируют переход на патент 
+ - Нет облачной кассы, платежи приходят на карту/расчетный счет, учет ведется вручную в Excel 
+ - Планируют расширение команды</t>
         </is>
       </c>
       <c r="R60" s="6" t="inlineStr">

</xml_diff>